<commit_message>
feat: improve dashboard drill-downs with detailed lists, footer summaries, and policy links
</commit_message>
<xml_diff>
--- a/production_demo.xlsx
+++ b/production_demo.xlsx
@@ -433,7 +433,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>CUST1001</v>
+        <v>CUST2001</v>
       </c>
       <c r="B2" t="str">
         <v>Rahul Verma</v>
@@ -448,7 +448,7 @@
         <v>AG1008</v>
       </c>
       <c r="F2" t="str">
-        <v>POL1001</v>
+        <v>POL2001</v>
       </c>
       <c r="G2" t="str">
         <v>RD1Y</v>
@@ -465,7 +465,7 @@
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>CUST1002</v>
+        <v>CUST2002</v>
       </c>
       <c r="B3" t="str">
         <v>Priya Sharma</v>
@@ -480,7 +480,7 @@
         <v>AG1000</v>
       </c>
       <c r="F3" t="str">
-        <v>POL1002</v>
+        <v>POL2002</v>
       </c>
       <c r="G3" t="str">
         <v>RD2Y</v>
@@ -497,7 +497,7 @@
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>CUST1003</v>
+        <v>CUST2003</v>
       </c>
       <c r="B4" t="str">
         <v>Amit Kumar</v>
@@ -512,7 +512,7 @@
         <v>AG1015</v>
       </c>
       <c r="F4" t="str">
-        <v>POL1003</v>
+        <v>POL2003</v>
       </c>
       <c r="G4" t="str">
         <v>PENS</v>
@@ -529,7 +529,7 @@
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>CUST1004</v>
+        <v>CUST2004</v>
       </c>
       <c r="B5" t="str">
         <v>Neha Gupta</v>
@@ -544,7 +544,7 @@
         <v>AG1008</v>
       </c>
       <c r="F5" t="str">
-        <v>POL1004</v>
+        <v>POL2004</v>
       </c>
       <c r="G5" t="str">
         <v>RD3Y</v>

</xml_diff>